<commit_message>
maj final en LATEX du rapport cas d usage (aled, c'etait vrm dur)
</commit_message>
<xml_diff>
--- a/Robot/Gyrobot_Component_Selection.xlsx
+++ b/Robot/Gyrobot_Component_Selection.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haasm\.gemini\antigravity\brain\1978af80-5a5c-4210-b052-21cb281392f5\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexv\Documents\Etude\POLYTECH\4AGPSE\Projet\depot_git\gyrobot_file\gyrobot\Robot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD391554-BD97-4BCC-92BD-1C8A1704C995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3C3010D-6120-4ECD-B690-467F1D38E551}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements" sheetId="1" r:id="rId1"/>
@@ -1379,9 +1379,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1389,12 +1388,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1429,6 +1423,42 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1732,1068 +1762,1069 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="109.7109375" customWidth="1"/>
-    <col min="2" max="2" width="24.7109375" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" customWidth="1"/>
-    <col min="4" max="4" width="78.140625" customWidth="1"/>
-    <col min="5" max="5" width="30.85546875" customWidth="1"/>
-    <col min="6" max="6" width="70.7109375" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" customWidth="1"/>
-    <col min="8" max="8" width="11.28515625" customWidth="1"/>
-    <col min="9" max="9" width="13" customWidth="1"/>
-    <col min="10" max="10" width="9.5703125" customWidth="1"/>
-    <col min="11" max="11" width="78" customWidth="1"/>
+    <col min="1" max="1" width="39.33203125" style="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.5546875" style="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="81.77734375" style="18" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32.21875" style="18" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="80.6640625" style="18" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.88671875" style="18" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.21875" style="18" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.88671875" style="18" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" style="18" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="82.88671875" style="18" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.109375" style="18"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:11" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="21" t="s">
         <v>378</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" s="22"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" s="31" t="s">
         <v>379</v>
       </c>
-      <c r="B4" s="26"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
-      <c r="H4" s="26"/>
-      <c r="I4" s="26"/>
-      <c r="J4" s="26"/>
-      <c r="K4" s="26"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="16" t="s">
+      <c r="B4" s="31"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
+      <c r="K4" s="31"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F5" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="16" t="s">
+      <c r="G5" s="17" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="23">
         <v>5</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="23">
         <v>10</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="18" t="s">
         <v>391</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="23">
         <v>2</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G8" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="23">
         <v>4</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="G10" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G12" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="4">
+      <c r="B14" s="23">
         <v>200</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="G14" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="G15" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="G16" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="G17" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="G18" s="3" t="s">
+      <c r="G18" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="G19" s="3" t="s">
+      <c r="G19" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="G20" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="G21" s="3" t="s">
+      <c r="G21" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A22" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="23" t="s">
         <v>74</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="G22" s="3" t="s">
+      <c r="G22" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="23" t="s">
         <v>78</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="23" t="s">
         <v>79</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="G23" s="3" t="s">
+      <c r="G23" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="23" t="s">
         <v>83</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F24" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="G24" s="3" t="s">
+      <c r="G24" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="23" t="s">
         <v>79</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="G25" s="3" t="s">
+      <c r="G25" s="32" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A28" s="26" t="s">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A28" s="31" t="s">
         <v>380</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="26"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="26"/>
-      <c r="G28" s="26"/>
-      <c r="H28" s="26"/>
-      <c r="I28" s="26"/>
-      <c r="J28" s="26"/>
-      <c r="K28" s="26"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A29" s="16" t="s">
+      <c r="B28" s="31"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="31"/>
+      <c r="G28" s="31"/>
+      <c r="H28" s="31"/>
+      <c r="I28" s="31"/>
+      <c r="J28" s="31"/>
+      <c r="K28" s="31"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A29" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="B29" s="16" t="s">
+      <c r="B29" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="C29" s="16" t="s">
+      <c r="C29" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="D29" s="16" t="s">
+      <c r="D29" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="E29" s="16" t="s">
+      <c r="E29" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="F29" s="16" t="s">
+      <c r="F29" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="G29" s="16" t="s">
+      <c r="G29" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="H29" s="16" t="s">
+      <c r="H29" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="I29" s="16" t="s">
+      <c r="I29" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="J29" s="16" t="s">
+      <c r="J29" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="K29" s="16" t="s">
+      <c r="K29" s="17" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A30" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="C30" s="4">
+      <c r="C30" s="23">
         <v>2</v>
       </c>
-      <c r="D30" s="4">
-        <v>0</v>
-      </c>
-      <c r="E30" s="4">
-        <v>0</v>
-      </c>
-      <c r="F30" s="4">
+      <c r="D30" s="23">
+        <v>0</v>
+      </c>
+      <c r="E30" s="23">
+        <v>0</v>
+      </c>
+      <c r="F30" s="23">
         <v>2</v>
       </c>
-      <c r="G30" s="4">
-        <v>0</v>
-      </c>
-      <c r="H30" s="4">
-        <v>0</v>
-      </c>
-      <c r="I30" s="4">
-        <v>0</v>
-      </c>
-      <c r="J30" s="4">
+      <c r="G30" s="23">
+        <v>0</v>
+      </c>
+      <c r="H30" s="23">
+        <v>0</v>
+      </c>
+      <c r="I30" s="23">
+        <v>0</v>
+      </c>
+      <c r="J30" s="23">
         <v>2</v>
       </c>
-      <c r="K30" t="s">
+      <c r="K30" s="18" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="C31" s="4">
+      <c r="C31" s="23">
         <v>2</v>
       </c>
-      <c r="D31" s="4">
-        <v>0</v>
-      </c>
-      <c r="E31" s="4">
-        <v>0</v>
-      </c>
-      <c r="F31" s="4">
+      <c r="D31" s="23">
+        <v>0</v>
+      </c>
+      <c r="E31" s="23">
+        <v>0</v>
+      </c>
+      <c r="F31" s="23">
         <v>2</v>
       </c>
-      <c r="G31" s="4">
-        <v>0</v>
-      </c>
-      <c r="H31" s="4">
-        <v>0</v>
-      </c>
-      <c r="I31" s="4">
-        <v>0</v>
-      </c>
-      <c r="J31" s="4">
+      <c r="G31" s="23">
+        <v>0</v>
+      </c>
+      <c r="H31" s="23">
+        <v>0</v>
+      </c>
+      <c r="I31" s="23">
+        <v>0</v>
+      </c>
+      <c r="J31" s="23">
         <v>2</v>
       </c>
-      <c r="K31" t="s">
+      <c r="K31" s="18" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="C32" s="4">
+      <c r="C32" s="23">
         <v>2</v>
       </c>
-      <c r="D32" s="4">
-        <v>0</v>
-      </c>
-      <c r="E32" s="4">
+      <c r="D32" s="23">
+        <v>0</v>
+      </c>
+      <c r="E32" s="23">
         <v>4</v>
       </c>
-      <c r="F32" s="4">
-        <v>0</v>
-      </c>
-      <c r="G32" s="4">
-        <v>0</v>
-      </c>
-      <c r="H32" s="4">
-        <v>0</v>
-      </c>
-      <c r="I32" s="4">
-        <v>0</v>
-      </c>
-      <c r="J32" s="4">
+      <c r="F32" s="23">
+        <v>0</v>
+      </c>
+      <c r="G32" s="23">
+        <v>0</v>
+      </c>
+      <c r="H32" s="23">
+        <v>0</v>
+      </c>
+      <c r="I32" s="23">
+        <v>0</v>
+      </c>
+      <c r="J32" s="23">
         <v>4</v>
       </c>
-      <c r="K32" t="s">
+      <c r="K32" s="18" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="C33" s="4">
+      <c r="C33" s="23">
         <v>1</v>
       </c>
-      <c r="D33" s="4">
-        <v>0</v>
-      </c>
-      <c r="E33" s="4">
-        <v>0</v>
-      </c>
-      <c r="F33" s="4">
-        <v>0</v>
-      </c>
-      <c r="G33" s="4">
+      <c r="D33" s="23">
+        <v>0</v>
+      </c>
+      <c r="E33" s="23">
+        <v>0</v>
+      </c>
+      <c r="F33" s="23">
+        <v>0</v>
+      </c>
+      <c r="G33" s="23">
         <v>2</v>
       </c>
-      <c r="H33" s="4">
-        <v>0</v>
-      </c>
-      <c r="I33" s="4">
-        <v>0</v>
-      </c>
-      <c r="J33" s="4">
+      <c r="H33" s="23">
+        <v>0</v>
+      </c>
+      <c r="I33" s="23">
+        <v>0</v>
+      </c>
+      <c r="J33" s="23">
         <v>2</v>
       </c>
-      <c r="K33" t="s">
+      <c r="K33" s="18" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A34" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="C34" s="4">
+      <c r="C34" s="23">
         <v>1</v>
       </c>
-      <c r="D34" s="4">
-        <v>0</v>
-      </c>
-      <c r="E34" s="4">
-        <v>0</v>
-      </c>
-      <c r="F34" s="4">
-        <v>0</v>
-      </c>
-      <c r="G34" s="4">
-        <v>0</v>
-      </c>
-      <c r="H34" s="4">
+      <c r="D34" s="23">
+        <v>0</v>
+      </c>
+      <c r="E34" s="23">
+        <v>0</v>
+      </c>
+      <c r="F34" s="23">
+        <v>0</v>
+      </c>
+      <c r="G34" s="23">
+        <v>0</v>
+      </c>
+      <c r="H34" s="23">
         <v>2</v>
       </c>
-      <c r="I34" s="4">
-        <v>0</v>
-      </c>
-      <c r="J34" s="4">
+      <c r="I34" s="23">
+        <v>0</v>
+      </c>
+      <c r="J34" s="23">
         <v>2</v>
       </c>
-      <c r="K34" t="s">
+      <c r="K34" s="18" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="C35" s="4">
+      <c r="C35" s="23">
         <v>1</v>
       </c>
-      <c r="D35" s="4">
+      <c r="D35" s="23">
         <v>1</v>
       </c>
-      <c r="E35" s="4">
-        <v>0</v>
-      </c>
-      <c r="F35" s="4">
-        <v>0</v>
-      </c>
-      <c r="G35" s="4">
-        <v>0</v>
-      </c>
-      <c r="H35" s="4">
-        <v>0</v>
-      </c>
-      <c r="I35" s="4">
-        <v>0</v>
-      </c>
-      <c r="J35" s="4">
+      <c r="E35" s="23">
+        <v>0</v>
+      </c>
+      <c r="F35" s="23">
+        <v>0</v>
+      </c>
+      <c r="G35" s="23">
+        <v>0</v>
+      </c>
+      <c r="H35" s="23">
+        <v>0</v>
+      </c>
+      <c r="I35" s="23">
+        <v>0</v>
+      </c>
+      <c r="J35" s="23">
         <v>1</v>
       </c>
-      <c r="K35" t="s">
+      <c r="K35" s="18" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="C36" s="4">
+      <c r="C36" s="23">
         <v>1</v>
       </c>
-      <c r="D36" s="4">
-        <v>0</v>
-      </c>
-      <c r="E36" s="4">
-        <v>0</v>
-      </c>
-      <c r="F36" s="4">
+      <c r="D36" s="23">
+        <v>0</v>
+      </c>
+      <c r="E36" s="23">
+        <v>0</v>
+      </c>
+      <c r="F36" s="23">
         <v>1</v>
       </c>
-      <c r="G36" s="4">
-        <v>0</v>
-      </c>
-      <c r="H36" s="4">
-        <v>0</v>
-      </c>
-      <c r="I36" s="4">
-        <v>0</v>
-      </c>
-      <c r="J36" s="4">
+      <c r="G36" s="23">
+        <v>0</v>
+      </c>
+      <c r="H36" s="23">
+        <v>0</v>
+      </c>
+      <c r="I36" s="23">
+        <v>0</v>
+      </c>
+      <c r="J36" s="23">
         <v>1</v>
       </c>
-      <c r="K36" t="s">
+      <c r="K36" s="18" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A37" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="C37" s="4">
+      <c r="C37" s="23">
         <v>1</v>
       </c>
-      <c r="D37" s="4">
-        <v>0</v>
-      </c>
-      <c r="E37" s="4">
-        <v>0</v>
-      </c>
-      <c r="F37" s="4">
-        <v>0</v>
-      </c>
-      <c r="G37" s="4">
-        <v>0</v>
-      </c>
-      <c r="H37" s="4">
+      <c r="D37" s="23">
+        <v>0</v>
+      </c>
+      <c r="E37" s="23">
+        <v>0</v>
+      </c>
+      <c r="F37" s="23">
+        <v>0</v>
+      </c>
+      <c r="G37" s="23">
+        <v>0</v>
+      </c>
+      <c r="H37" s="23">
         <v>2</v>
       </c>
-      <c r="I37" s="4">
-        <v>0</v>
-      </c>
-      <c r="J37" s="4">
+      <c r="I37" s="23">
+        <v>0</v>
+      </c>
+      <c r="J37" s="23">
         <v>2</v>
       </c>
-      <c r="K37" t="s">
+      <c r="K37" s="18" t="s">
         <v>396</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="C38" s="4">
+      <c r="C38" s="23">
         <v>1</v>
       </c>
-      <c r="D38" s="4">
-        <v>0</v>
-      </c>
-      <c r="E38" s="4">
-        <v>0</v>
-      </c>
-      <c r="F38" s="4">
-        <v>0</v>
-      </c>
-      <c r="G38" s="4">
-        <v>0</v>
-      </c>
-      <c r="H38" s="4">
-        <v>0</v>
-      </c>
-      <c r="I38" s="4">
+      <c r="D38" s="23">
+        <v>0</v>
+      </c>
+      <c r="E38" s="23">
+        <v>0</v>
+      </c>
+      <c r="F38" s="23">
+        <v>0</v>
+      </c>
+      <c r="G38" s="23">
+        <v>0</v>
+      </c>
+      <c r="H38" s="23">
+        <v>0</v>
+      </c>
+      <c r="I38" s="23">
         <v>1</v>
       </c>
-      <c r="J38" s="4">
+      <c r="J38" s="23">
         <v>1</v>
       </c>
-      <c r="K38" t="s">
+      <c r="K38" s="18" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="C39" s="4">
+      <c r="C39" s="23">
         <v>1</v>
       </c>
-      <c r="D39" s="4">
-        <v>0</v>
-      </c>
-      <c r="E39" s="4">
-        <v>0</v>
-      </c>
-      <c r="F39" s="4">
-        <v>0</v>
-      </c>
-      <c r="G39" s="4">
-        <v>0</v>
-      </c>
-      <c r="H39" s="4">
+      <c r="D39" s="23">
+        <v>0</v>
+      </c>
+      <c r="E39" s="23">
+        <v>0</v>
+      </c>
+      <c r="F39" s="23">
+        <v>0</v>
+      </c>
+      <c r="G39" s="23">
+        <v>0</v>
+      </c>
+      <c r="H39" s="23">
         <v>2</v>
       </c>
-      <c r="I39" s="4">
-        <v>0</v>
-      </c>
-      <c r="J39" s="4">
+      <c r="I39" s="23">
+        <v>0</v>
+      </c>
+      <c r="J39" s="23">
         <v>2</v>
       </c>
-      <c r="K39" t="s">
+      <c r="K39" s="18" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A42" s="26" t="s">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42" s="31" t="s">
         <v>377</v>
       </c>
-      <c r="B42" s="26"/>
-      <c r="C42" s="26"/>
-      <c r="D42" s="26"/>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A43" s="16" t="s">
+      <c r="B42" s="31"/>
+      <c r="C42" s="31"/>
+      <c r="D42" s="31"/>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="B43" s="16" t="s">
+      <c r="B43" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="C43" s="16" t="s">
+      <c r="C43" s="17" t="s">
         <v>120</v>
       </c>
-      <c r="D43" s="16" t="s">
+      <c r="D43" s="17" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C44" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D44" s="18" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C45" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D45" t="s">
+      <c r="D45" s="18" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46" s="18" t="s">
         <v>128</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C46" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D46" t="s">
+      <c r="D46" s="18" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C47" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="D47" t="s">
+      <c r="D47" s="18" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B48" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C48" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D48" s="18" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="18" t="s">
         <v>395</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C49" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="D49" t="s">
+      <c r="D49" s="18" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C50" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="D50" t="s">
+      <c r="D50" s="18" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="18" t="s">
         <v>142</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C51" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="D51" t="s">
+      <c r="D51" s="18" t="s">
         <v>144</v>
       </c>
     </row>
@@ -2811,518 +2842,519 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" customWidth="1"/>
-    <col min="2" max="2" width="41" customWidth="1"/>
-    <col min="3" max="3" width="44.5703125" customWidth="1"/>
-    <col min="4" max="4" width="46.5703125" customWidth="1"/>
-    <col min="5" max="5" width="240.5703125" customWidth="1"/>
-    <col min="6" max="6" width="255" customWidth="1"/>
-    <col min="7" max="7" width="39.140625" customWidth="1"/>
-    <col min="8" max="8" width="74" customWidth="1"/>
-    <col min="9" max="9" width="4.140625" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="13" customWidth="1"/>
-    <col min="12" max="12" width="22.85546875" customWidth="1"/>
+    <col min="1" max="1" width="4.109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23" style="18" customWidth="1"/>
+    <col min="3" max="3" width="20" style="18" customWidth="1"/>
+    <col min="4" max="4" width="23.88671875" style="18" customWidth="1"/>
+    <col min="5" max="5" width="100" style="18" customWidth="1"/>
+    <col min="6" max="6" width="135.77734375" style="18" customWidth="1"/>
+    <col min="7" max="7" width="26.77734375" style="18" customWidth="1"/>
+    <col min="8" max="8" width="60.6640625" style="18" customWidth="1"/>
+    <col min="9" max="9" width="4.21875" style="18" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.109375" style="18" customWidth="1"/>
+    <col min="11" max="11" width="12.109375" style="18" customWidth="1"/>
+    <col min="12" max="12" width="20.88671875" style="18" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="9.109375" style="18"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:12" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="21" t="s">
         <v>373</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" s="22"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" s="17" t="s">
         <v>145</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="17" t="s">
         <v>146</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="17" t="s">
         <v>148</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="17" t="s">
         <v>149</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="17" t="s">
         <v>374</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="17" t="s">
         <v>150</v>
       </c>
-      <c r="H4" s="16" t="s">
+      <c r="H4" s="17" t="s">
         <v>151</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="I4" s="17" t="s">
         <v>152</v>
       </c>
-      <c r="J4" s="16" t="s">
+      <c r="J4" s="17" t="s">
         <v>153</v>
       </c>
-      <c r="K4" s="16" t="s">
+      <c r="K4" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="L4" s="16" t="s">
+      <c r="L4" s="17" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="4">
+    <row r="5" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="23">
         <v>1</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="18" t="s">
         <v>387</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="G5" s="24" t="s">
+      <c r="G5" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="H5" s="24" t="s">
+      <c r="H5" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="I5" s="4">
+      <c r="I5" s="23">
         <v>1</v>
       </c>
-      <c r="J5" s="5">
+      <c r="J5" s="24">
         <v>216</v>
       </c>
-      <c r="K5" s="5">
-        <v>0</v>
-      </c>
-      <c r="L5" s="6" t="s">
+      <c r="K5" s="24">
+        <v>0</v>
+      </c>
+      <c r="L5" s="25" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="4">
+    <row r="6" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="23">
         <v>2</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="18" t="s">
         <v>388</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="18" t="s">
         <v>165</v>
       </c>
-      <c r="G6" s="24" t="s">
+      <c r="G6" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="H6" s="24" t="s">
+      <c r="H6" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="I6" s="4">
+      <c r="I6" s="23">
         <v>1</v>
       </c>
-      <c r="J6" s="5">
+      <c r="J6" s="24">
         <v>11.9</v>
       </c>
-      <c r="K6" s="5">
-        <v>0</v>
-      </c>
-      <c r="L6" s="6" t="s">
+      <c r="K6" s="24">
+        <v>0</v>
+      </c>
+      <c r="L6" s="25" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="4">
+    <row r="7" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="23">
         <v>3</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="18" t="s">
         <v>171</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="18" t="s">
         <v>172</v>
       </c>
-      <c r="G7" s="24" t="s">
+      <c r="G7" s="18" t="s">
         <v>173</v>
       </c>
-      <c r="H7" s="24" t="s">
+      <c r="H7" s="18" t="s">
         <v>174</v>
       </c>
-      <c r="I7" s="4">
+      <c r="I7" s="23">
         <v>1</v>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="24">
         <v>83.9</v>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="24">
         <v>83.9</v>
       </c>
-      <c r="L7" s="7" t="s">
+      <c r="L7" s="26" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="4">
+    <row r="8" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="23">
         <v>4</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="18" t="s">
         <v>176</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="18" t="s">
         <v>178</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="18" t="s">
         <v>180</v>
       </c>
-      <c r="G8" s="24" t="s">
+      <c r="G8" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="H8" s="24" t="s">
+      <c r="H8" s="18" t="s">
         <v>182</v>
       </c>
-      <c r="I8" s="4">
+      <c r="I8" s="23">
         <v>1</v>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="24">
         <v>14.5</v>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="24">
         <v>14.5</v>
       </c>
-      <c r="L8" s="7" t="s">
+      <c r="L8" s="26" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="45" x14ac:dyDescent="0.25">
-      <c r="A9" s="4">
+    <row r="9" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="23">
         <v>5</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="18" t="s">
         <v>183</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="18" t="s">
         <v>185</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="G9" s="24" t="s">
+      <c r="G9" s="18" t="s">
         <v>188</v>
       </c>
-      <c r="H9" s="24" t="s">
+      <c r="H9" s="18" t="s">
         <v>189</v>
       </c>
-      <c r="I9" s="4">
+      <c r="I9" s="23">
         <v>2</v>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="24">
         <v>21.5</v>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="24">
         <v>43</v>
       </c>
-      <c r="L9" s="7" t="s">
+      <c r="L9" s="26" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="4">
+    <row r="10" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="23">
         <v>6</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="18" t="s">
         <v>190</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="18" t="s">
         <v>192</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="G10" s="24" t="s">
+      <c r="G10" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="H10" s="24" t="s">
+      <c r="H10" s="18" t="s">
         <v>196</v>
       </c>
-      <c r="I10" s="4">
+      <c r="I10" s="23">
         <v>1</v>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="24">
         <v>29.2</v>
       </c>
-      <c r="K10" s="5">
+      <c r="K10" s="24">
         <v>29.2</v>
       </c>
-      <c r="L10" s="7" t="s">
+      <c r="L10" s="26" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="4">
+    <row r="11" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="23">
         <v>7</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="18" t="s">
         <v>197</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="18" t="s">
         <v>198</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="18" t="s">
         <v>199</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="18" t="s">
         <v>389</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="18" t="s">
         <v>200</v>
       </c>
-      <c r="G11" s="24" t="s">
+      <c r="G11" s="18" t="s">
         <v>201</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11" s="18" t="s">
         <v>202</v>
       </c>
-      <c r="I11" s="4">
+      <c r="I11" s="23">
         <v>1</v>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="24">
         <v>29.9</v>
       </c>
-      <c r="K11" s="5">
-        <v>0</v>
-      </c>
-      <c r="L11" s="6" t="s">
+      <c r="K11" s="24">
+        <v>0</v>
+      </c>
+      <c r="L11" s="25" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="4">
+    <row r="12" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="23">
         <v>8</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="18" t="s">
         <v>203</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="18" t="s">
         <v>205</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="18" t="s">
         <v>206</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="18" t="s">
         <v>207</v>
       </c>
-      <c r="G12" s="24" t="s">
+      <c r="G12" s="18" t="s">
         <v>208</v>
       </c>
-      <c r="H12" t="s">
+      <c r="H12" s="18" t="s">
         <v>209</v>
       </c>
-      <c r="I12" s="4">
+      <c r="I12" s="23">
         <v>1</v>
       </c>
-      <c r="J12" s="5">
+      <c r="J12" s="24">
         <v>1.6</v>
       </c>
-      <c r="K12" s="5">
+      <c r="K12" s="24">
         <v>1.6</v>
       </c>
-      <c r="L12" s="7" t="s">
+      <c r="L12" s="26" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="45" x14ac:dyDescent="0.25">
-      <c r="A13" s="4">
+    <row r="13" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="23">
         <v>9</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="18" t="s">
         <v>210</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="18" t="s">
         <v>211</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="18" t="s">
         <v>212</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="18" t="s">
         <v>213</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="18" t="s">
         <v>214</v>
       </c>
-      <c r="G13" s="24" t="s">
+      <c r="G13" s="18" t="s">
         <v>215</v>
       </c>
-      <c r="H13" s="24" t="s">
+      <c r="H13" s="18" t="s">
         <v>216</v>
       </c>
-      <c r="I13" s="4">
+      <c r="I13" s="23">
         <v>2</v>
       </c>
-      <c r="J13" s="5">
-        <v>0</v>
-      </c>
-      <c r="K13" s="5">
-        <v>0</v>
-      </c>
-      <c r="L13" s="8" t="s">
+      <c r="J13" s="24">
+        <v>0</v>
+      </c>
+      <c r="K13" s="24">
+        <v>0</v>
+      </c>
+      <c r="L13" s="27" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="4">
+    <row r="14" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="23">
         <v>10</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="18" t="s">
         <v>217</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="18" t="s">
         <v>218</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="18" t="s">
         <v>219</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="18" t="s">
         <v>220</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="18" t="s">
         <v>221</v>
       </c>
-      <c r="G14" s="24" t="s">
+      <c r="G14" s="18" t="s">
         <v>222</v>
       </c>
-      <c r="H14" s="24" t="s">
+      <c r="H14" s="18" t="s">
         <v>223</v>
       </c>
-      <c r="I14" s="4">
+      <c r="I14" s="23">
         <v>1</v>
       </c>
-      <c r="J14" s="5">
+      <c r="J14" s="24">
         <v>9.6999999999999993</v>
       </c>
-      <c r="K14" s="5">
+      <c r="K14" s="24">
         <v>9.6999999999999993</v>
       </c>
-      <c r="L14" s="7" t="s">
+      <c r="L14" s="26" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="45" x14ac:dyDescent="0.25">
-      <c r="A15" s="4">
+    <row r="15" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A15" s="23">
         <v>11</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="18" t="s">
         <v>225</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="18" t="s">
         <v>226</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="18" t="s">
         <v>227</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="18" t="s">
         <v>228</v>
       </c>
-      <c r="G15" s="24" t="s">
+      <c r="G15" s="18" t="s">
         <v>229</v>
       </c>
-      <c r="H15" s="24" t="s">
+      <c r="H15" s="18" t="s">
         <v>230</v>
       </c>
-      <c r="I15" s="4">
+      <c r="I15" s="23">
         <v>1</v>
       </c>
-      <c r="J15" s="5">
+      <c r="J15" s="24">
         <v>29.9</v>
       </c>
-      <c r="K15" s="5">
-        <v>0</v>
-      </c>
-      <c r="L15" s="6" t="s">
+      <c r="K15" s="24">
+        <v>0</v>
+      </c>
+      <c r="L15" s="25" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16" s="9"/>
-      <c r="B16" s="1" t="s">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A16" s="28"/>
+      <c r="B16" s="29" t="s">
         <v>383</v>
       </c>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="1">
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
+      <c r="G16" s="28"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="29">
         <f>SUM(I5:I15)</f>
         <v>13</v>
       </c>
-      <c r="J16" s="9"/>
-      <c r="K16" s="10">
+      <c r="J16" s="28"/>
+      <c r="K16" s="30">
         <f>SUM(K5:K15)</f>
         <v>181.89999999999998</v>
       </c>
-      <c r="L16" s="9"/>
+      <c r="L16" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3335,63 +3367,63 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="83.85546875" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" customWidth="1"/>
-    <col min="3" max="3" width="31.28515625" customWidth="1"/>
-    <col min="4" max="4" width="35.28515625" customWidth="1"/>
+    <col min="1" max="1" width="83.88671875" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" customWidth="1"/>
+    <col min="3" max="3" width="31.33203125" customWidth="1"/>
+    <col min="4" max="4" width="35.33203125" customWidth="1"/>
     <col min="5" max="5" width="28" customWidth="1"/>
-    <col min="6" max="6" width="35.42578125" customWidth="1"/>
-    <col min="7" max="7" width="9.140625" customWidth="1"/>
+    <col min="6" max="6" width="35.44140625" customWidth="1"/>
+    <col min="7" max="7" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="19" t="s">
         <v>366</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="20" t="s">
         <v>397</v>
       </c>
-      <c r="B4" s="26"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
         <v>231</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="17" t="s">
         <v>367</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="10" t="s">
         <v>368</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="10" t="s">
         <v>369</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F5" s="10" t="s">
         <v>370</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>232</v>
       </c>
@@ -3411,7 +3443,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>237</v>
       </c>
@@ -3431,7 +3463,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>242</v>
       </c>
@@ -3451,7 +3483,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>248</v>
       </c>
@@ -3471,7 +3503,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>253</v>
       </c>
@@ -3491,162 +3523,162 @@
         <v>257</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>258</v>
       </c>
       <c r="B11" t="s">
         <v>243</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="5" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>261</v>
       </c>
       <c r="B12" t="s">
         <v>243</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="F12" s="6" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>263</v>
       </c>
       <c r="B13" t="s">
         <v>243</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="4" t="s">
         <v>372</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="4" t="s">
         <v>372</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="4" t="s">
         <v>372</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="5" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>264</v>
       </c>
       <c r="B14" t="s">
         <v>243</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="E14" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="F14" s="11" t="s">
+      <c r="F14" s="5" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B17" s="13"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B18" s="13"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B19" s="13"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="13"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="13"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B22" s="13"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B23" s="13"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="12"/>
-      <c r="B24" s="12"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="12"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="12"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="12"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="12"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="15"/>
-      <c r="F28" s="15"/>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B17" s="7"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B18" s="7"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B19" s="7"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B20" s="7"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B21" s="7"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B22" s="7"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B23" s="7"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="6"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="6"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="6"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="6"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3660,720 +3692,720 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="78" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" customWidth="1"/>
-    <col min="3" max="3" width="21.5703125" style="4" customWidth="1"/>
-    <col min="4" max="4" width="77.5703125" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" customWidth="1"/>
+    <col min="3" max="3" width="21.5546875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="77.5546875" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
-    <col min="6" max="6" width="11.85546875" customWidth="1"/>
-    <col min="7" max="7" width="85.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.88671875" customWidth="1"/>
+    <col min="7" max="7" width="85.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="19" t="s">
         <v>365</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="20" t="s">
         <v>268</v>
       </c>
-      <c r="B4" s="26"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
         <v>269</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="10" t="s">
         <v>270</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="10" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>272</v>
       </c>
-      <c r="B6" s="18">
+      <c r="B6" s="12">
         <v>11.1</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>84</v>
       </c>
       <c r="D6" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>274</v>
       </c>
-      <c r="B7" s="18">
+      <c r="B7" s="12">
         <v>12.6</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>84</v>
       </c>
       <c r="D7" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>276</v>
       </c>
-      <c r="B8" s="18">
+      <c r="B8" s="12">
         <v>9.9</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>84</v>
       </c>
       <c r="D8" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>278</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="3">
         <v>2700</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>279</v>
       </c>
       <c r="D9" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>281</v>
       </c>
-      <c r="B10" s="18">
+      <c r="B10" s="12">
         <v>29.97</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>282</v>
       </c>
       <c r="D10" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>284</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B11" s="3">
         <v>30</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>285</v>
       </c>
       <c r="D11" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>287</v>
       </c>
-      <c r="B12" s="21">
+      <c r="B12" s="15">
         <v>0.8</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="3" t="s">
         <v>243</v>
       </c>
       <c r="D12" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>289</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B13" s="3">
         <v>2160</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="3" t="s">
         <v>279</v>
       </c>
       <c r="D13" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>291</v>
       </c>
-      <c r="B14" s="18">
+      <c r="B14" s="12">
         <v>5</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="3" t="s">
         <v>84</v>
       </c>
       <c r="D14" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>293</v>
       </c>
-      <c r="B15" s="21">
+      <c r="B15" s="15">
         <v>0.88</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="3" t="s">
         <v>243</v>
       </c>
       <c r="D15" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>294</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B16" s="3">
         <v>5000</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="3" t="s">
         <v>295</v>
       </c>
       <c r="D16" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="26" t="s">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="20" t="s">
         <v>297</v>
       </c>
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="16" t="s">
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="B20" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="C20" s="16" t="s">
+      <c r="C20" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="D20" s="16" t="s">
+      <c r="D20" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="E20" s="16" t="s">
+      <c r="E20" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="F20" s="16" t="s">
+      <c r="F20" s="10" t="s">
         <v>302</v>
       </c>
-      <c r="G20" s="16" t="s">
+      <c r="G20" s="10" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>304</v>
       </c>
-      <c r="B21" s="4">
+      <c r="B21" s="3">
         <v>1</v>
       </c>
-      <c r="C21" s="22" t="s">
+      <c r="C21" s="16" t="s">
         <v>305</v>
       </c>
-      <c r="D21" s="17">
+      <c r="D21" s="11">
         <v>1550</v>
       </c>
-      <c r="E21" s="17">
+      <c r="E21" s="11">
         <v>1550</v>
       </c>
-      <c r="F21" s="17">
+      <c r="F21" s="11">
         <v>7750</v>
       </c>
       <c r="G21" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>307</v>
       </c>
-      <c r="B22" s="4">
+      <c r="B22" s="3">
         <v>1</v>
       </c>
-      <c r="C22" s="22" t="s">
+      <c r="C22" s="16" t="s">
         <v>305</v>
       </c>
-      <c r="D22" s="17">
+      <c r="D22" s="11">
         <v>230</v>
       </c>
-      <c r="E22" s="17">
+      <c r="E22" s="11">
         <v>230</v>
       </c>
-      <c r="F22" s="17">
+      <c r="F22" s="11">
         <v>1150</v>
       </c>
       <c r="G22" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>309</v>
       </c>
-      <c r="B23" s="4">
+      <c r="B23" s="3">
         <v>1</v>
       </c>
-      <c r="C23" s="22" t="s">
+      <c r="C23" s="16" t="s">
         <v>310</v>
       </c>
-      <c r="D23" s="17">
+      <c r="D23" s="11">
         <v>180</v>
       </c>
-      <c r="E23" s="17">
+      <c r="E23" s="11">
         <v>180</v>
       </c>
-      <c r="F23" s="17">
+      <c r="F23" s="11">
         <v>900</v>
       </c>
       <c r="G23" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>312</v>
       </c>
-      <c r="B24" s="4">
+      <c r="B24" s="3">
         <v>1</v>
       </c>
-      <c r="C24" s="22" t="s">
+      <c r="C24" s="16" t="s">
         <v>305</v>
       </c>
-      <c r="D24" s="17">
+      <c r="D24" s="11">
         <v>70</v>
       </c>
-      <c r="E24" s="17">
+      <c r="E24" s="11">
         <v>70</v>
       </c>
-      <c r="F24" s="17">
+      <c r="F24" s="11">
         <v>350</v>
       </c>
       <c r="G24" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>314</v>
       </c>
-      <c r="B25" s="4">
+      <c r="B25" s="3">
         <v>1</v>
       </c>
-      <c r="C25" s="22" t="s">
+      <c r="C25" s="16" t="s">
         <v>305</v>
       </c>
-      <c r="D25" s="17">
+      <c r="D25" s="11">
         <v>1</v>
       </c>
-      <c r="E25" s="17">
+      <c r="E25" s="11">
         <v>1</v>
       </c>
-      <c r="F25" s="17">
+      <c r="F25" s="11">
         <v>5</v>
       </c>
       <c r="G25" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>315</v>
       </c>
-      <c r="B26" s="4">
+      <c r="B26" s="3">
         <v>1</v>
       </c>
-      <c r="C26" s="22" t="s">
+      <c r="C26" s="16" t="s">
         <v>305</v>
       </c>
-      <c r="D26" s="17">
+      <c r="D26" s="11">
         <v>5</v>
       </c>
-      <c r="E26" s="17">
+      <c r="E26" s="11">
         <v>5</v>
       </c>
-      <c r="F26" s="17">
+      <c r="F26" s="11">
         <v>25</v>
       </c>
       <c r="G26" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>317</v>
       </c>
-      <c r="B27" s="4">
+      <c r="B27" s="3">
         <v>2</v>
       </c>
-      <c r="C27" s="22" t="s">
+      <c r="C27" s="16" t="s">
         <v>318</v>
       </c>
-      <c r="D27" s="17">
+      <c r="D27" s="11">
         <v>160</v>
       </c>
-      <c r="E27" s="17">
+      <c r="E27" s="11">
         <v>320</v>
       </c>
-      <c r="F27" s="17">
+      <c r="F27" s="11">
         <v>3552</v>
       </c>
       <c r="G27" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>319</v>
       </c>
-      <c r="B28" s="4">
+      <c r="B28" s="3">
         <v>2</v>
       </c>
-      <c r="C28" s="22" t="s">
+      <c r="C28" s="16" t="s">
         <v>318</v>
       </c>
-      <c r="D28" s="17">
+      <c r="D28" s="11">
         <v>260</v>
       </c>
-      <c r="E28" s="17">
+      <c r="E28" s="11">
         <v>520</v>
       </c>
-      <c r="F28" s="17">
+      <c r="F28" s="11">
         <v>5772</v>
       </c>
       <c r="G28" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>321</v>
       </c>
-      <c r="B29" s="4">
+      <c r="B29" s="3">
         <v>2</v>
       </c>
-      <c r="C29" s="22" t="s">
+      <c r="C29" s="16" t="s">
         <v>318</v>
       </c>
-      <c r="D29" s="17">
+      <c r="D29" s="11">
         <v>550</v>
       </c>
-      <c r="E29" s="17">
+      <c r="E29" s="11">
         <v>1100</v>
       </c>
-      <c r="F29" s="17">
+      <c r="F29" s="11">
         <v>12210</v>
       </c>
       <c r="G29" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="26" t="s">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" s="20" t="s">
         <v>398</v>
       </c>
-      <c r="B32" s="26"/>
-      <c r="C32" s="26"/>
-      <c r="D32" s="26"/>
-      <c r="E32" s="26"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="16" t="s">
+      <c r="B32" s="20"/>
+      <c r="C32" s="20"/>
+      <c r="D32" s="20"/>
+      <c r="E32" s="20"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="10" t="s">
         <v>323</v>
       </c>
-      <c r="B33" s="16" t="s">
+      <c r="B33" s="10" t="s">
         <v>270</v>
       </c>
-      <c r="C33" s="16" t="s">
+      <c r="C33" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D33" s="16" t="s">
+      <c r="D33" s="10" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>324</v>
       </c>
-      <c r="B34" s="17">
+      <c r="B34" s="11">
         <v>2036</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="3" t="s">
         <v>295</v>
       </c>
       <c r="D34" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>326</v>
       </c>
-      <c r="B35" s="18">
+      <c r="B35" s="12">
         <v>10.18</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C35" s="3" t="s">
         <v>327</v>
       </c>
       <c r="D35" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>329</v>
       </c>
-      <c r="B36" s="17">
+      <c r="B36" s="11">
         <v>1042</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="C36" s="3" t="s">
         <v>295</v>
       </c>
       <c r="D36" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>331</v>
       </c>
-      <c r="B37" s="17">
+      <c r="B37" s="11">
         <v>320</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="C37" s="3" t="s">
         <v>295</v>
       </c>
       <c r="D37" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>333</v>
       </c>
-      <c r="B38" s="17">
+      <c r="B38" s="11">
         <v>1362</v>
       </c>
-      <c r="C38" s="4" t="s">
+      <c r="C38" s="3" t="s">
         <v>295</v>
       </c>
       <c r="D38" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>335</v>
       </c>
-      <c r="B39" s="18">
+      <c r="B39" s="12">
         <v>15.12</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="C39" s="3" t="s">
         <v>327</v>
       </c>
       <c r="D39" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>337</v>
       </c>
-      <c r="B40" s="19">
+      <c r="B40" s="13">
         <v>1.5860000000000001</v>
       </c>
-      <c r="C40" s="4" t="s">
+      <c r="C40" s="3" t="s">
         <v>338</v>
       </c>
       <c r="D40" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>340</v>
       </c>
-      <c r="B41" s="17">
+      <c r="B41" s="11">
         <v>1562</v>
       </c>
-      <c r="C41" s="4" t="s">
+      <c r="C41" s="3" t="s">
         <v>295</v>
       </c>
       <c r="D41" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>342</v>
       </c>
-      <c r="B42" s="18">
+      <c r="B42" s="12">
         <v>17.34</v>
       </c>
-      <c r="C42" s="4" t="s">
+      <c r="C42" s="3" t="s">
         <v>327</v>
       </c>
       <c r="D42" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>344</v>
       </c>
-      <c r="B43" s="19">
+      <c r="B43" s="13">
         <v>1.383</v>
       </c>
-      <c r="C43" s="4" t="s">
+      <c r="C43" s="3" t="s">
         <v>338</v>
       </c>
       <c r="D43" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>346</v>
       </c>
-      <c r="B44" s="17">
+      <c r="B44" s="11">
         <v>2142</v>
       </c>
-      <c r="C44" s="4" t="s">
+      <c r="C44" s="3" t="s">
         <v>295</v>
       </c>
       <c r="D44" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>348</v>
       </c>
-      <c r="B45" s="19">
+      <c r="B45" s="13">
         <v>1.008</v>
       </c>
-      <c r="C45" s="4" t="s">
+      <c r="C45" s="3" t="s">
         <v>338</v>
       </c>
       <c r="D45" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>350</v>
       </c>
-      <c r="B46" s="4" t="s">
+      <c r="B46" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C46" s="4" t="s">
+      <c r="C46" s="3" t="s">
         <v>79</v>
       </c>
       <c r="D46" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>352</v>
       </c>
-      <c r="B47" s="3" t="s">
+      <c r="B47" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C47" s="4" t="s">
+      <c r="C47" s="3" t="s">
         <v>243</v>
       </c>
       <c r="D47" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>354</v>
       </c>
-      <c r="B48" s="17">
+      <c r="B48" s="11">
         <v>5000</v>
       </c>
-      <c r="C48" s="4" t="s">
+      <c r="C48" s="3" t="s">
         <v>295</v>
       </c>
       <c r="D48" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>356</v>
       </c>
-      <c r="B49" s="20">
+      <c r="B49" s="14">
         <v>59.3</v>
       </c>
-      <c r="C49" s="4" t="s">
+      <c r="C49" s="3" t="s">
         <v>357</v>
       </c>
       <c r="D49" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>359</v>
       </c>
-      <c r="B50" s="18">
+      <c r="B50" s="12">
         <v>4.9000000000000004</v>
       </c>
-      <c r="C50" s="4" t="s">
+      <c r="C50" s="3" t="s">
         <v>84</v>
       </c>
       <c r="D50" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>361</v>
       </c>
-      <c r="B51" s="3" t="s">
+      <c r="B51" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="C51" s="4" t="s">
+      <c r="C51" s="3" t="s">
         <v>243</v>
       </c>
       <c r="D51" t="s">

</xml_diff>